<commit_message>
Doc(JDT)Remplissage du journal de travail
</commit_message>
<xml_diff>
--- a/Doc/Journal-de-Travail_BamertMathieu.xlsx
+++ b/Doc/Journal-de-Travail_BamertMathieu.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pv23aha\Documents\GitHub\P_321_BitRuisseau\Doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mathi\OneDrive\Documents\GitHub\P_321_BitRuisseau\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A47660B1-915E-400F-8AFB-E6010C9108F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C41C2708-479B-4F16-AFB1-EE565F307EC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="64">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -213,6 +213,27 @@
   <si>
     <t>Rajout de la classe basicsong</t>
   </si>
+  <si>
+    <t>Changement du nom de fichier</t>
+  </si>
+  <si>
+    <t>Création du protocole mqtt</t>
+  </si>
+  <si>
+    <t>Modification du design</t>
+  </si>
+  <si>
+    <t>Modification du code pour avoir que des méthodes courte</t>
+  </si>
+  <si>
+    <t>Faire que les datagridview se remplis quand je choissis un dossier mp3</t>
+  </si>
+  <si>
+    <t>Restructuration du code et refais une grande partie du code pour qu'on puissent me voir en ligne sur le brocker</t>
+  </si>
+  <si>
+    <t>Améliorer tout le code pour qu'ils soit plus compréhensible</t>
+  </si>
 </sst>
 </file>
 
@@ -225,7 +246,7 @@
     <numFmt numFmtId="167" formatCode="dd\ mmm"/>
     <numFmt numFmtId="168" formatCode="00\ &quot;min&quot;"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -361,6 +382,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFF0F6FC"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="14">
     <fill>
@@ -490,10 +525,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -685,6 +721,10 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="16" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
@@ -695,12 +735,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="18">
@@ -1244,16 +1285,16 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>725</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>225</c:v>
+                  <c:v>245</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>45</c:v>
+                  <c:v>135</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1317,6 +1358,7 @@
     </c:legend>
     <c:plotVisOnly val="0"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1324,7 +1366,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1664,6 +1705,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1671,7 +1713,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2099,13 +2140,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.64935064935064934</c:v>
+                  <c:v>0.65610859728506787</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.29220779220779219</c:v>
+                  <c:v>0.22171945701357465</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2260,6 +2301,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2267,7 +2309,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4317,15 +4358,15 @@
       <c r="G1" s="11"/>
     </row>
     <row r="2" spans="1:15" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A2" s="87" t="s">
+      <c r="A2" s="88" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="87"/>
-      <c r="C2" s="85" t="s">
+      <c r="B2" s="88"/>
+      <c r="C2" s="86" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
+      <c r="D2" s="86"/>
+      <c r="E2" s="86"/>
       <c r="F2" s="5" t="s">
         <v>2</v>
       </c>
@@ -4334,13 +4375,13 @@
       </c>
     </row>
     <row r="3" spans="1:15" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A3" s="87" t="s">
+      <c r="A3" s="88" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="87"/>
+      <c r="B3" s="88"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>12 heures 50 minutes</v>
+        <v>18 heures 25 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4353,24 +4394,24 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>180</v>
+        <v>300</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>590</v>
+        <v>805</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>770</v>
+        <v>1105</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="C5" s="86" t="s">
+      <c r="C5" s="87" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="86"/>
+      <c r="D5" s="87"/>
     </row>
     <row r="6" spans="1:15" s="15" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
@@ -4991,7 +5032,7 @@
       <c r="E32" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="F32" s="88" t="s">
+      <c r="F32" s="85" t="s">
         <v>54</v>
       </c>
       <c r="G32" s="39"/>
@@ -5045,11 +5086,15 @@
         <v>46003</v>
       </c>
       <c r="C35" s="35"/>
-      <c r="D35" s="36"/>
+      <c r="D35" s="36">
+        <v>15</v>
+      </c>
       <c r="E35" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="F35" s="23"/>
+      <c r="F35" s="23" t="s">
+        <v>57</v>
+      </c>
       <c r="G35" s="40"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -5061,11 +5106,15 @@
         <v>46003</v>
       </c>
       <c r="C36" s="31"/>
-      <c r="D36" s="32"/>
+      <c r="D36" s="32">
+        <v>20</v>
+      </c>
       <c r="E36" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="F36" s="22"/>
+      <c r="F36" s="22" t="s">
+        <v>58</v>
+      </c>
       <c r="G36" s="39"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
@@ -5077,11 +5126,15 @@
         <v>46003</v>
       </c>
       <c r="C37" s="35"/>
-      <c r="D37" s="36"/>
+      <c r="D37" s="36">
+        <v>15</v>
+      </c>
       <c r="E37" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="F37" s="22"/>
+      <c r="F37" s="22" t="s">
+        <v>59</v>
+      </c>
       <c r="G37" s="40"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
@@ -5093,11 +5146,15 @@
         <v>46003</v>
       </c>
       <c r="C38" s="31"/>
-      <c r="D38" s="32"/>
+      <c r="D38" s="32">
+        <v>10</v>
+      </c>
       <c r="E38" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="F38" s="22"/>
+      <c r="F38" s="89" t="s">
+        <v>60</v>
+      </c>
       <c r="G38" s="39"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
@@ -5109,11 +5166,15 @@
         <v>46003</v>
       </c>
       <c r="C39" s="35"/>
-      <c r="D39" s="36"/>
+      <c r="D39" s="36">
+        <v>5</v>
+      </c>
       <c r="E39" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="F39" s="22"/>
+      <c r="F39" s="22" t="s">
+        <v>30</v>
+      </c>
       <c r="G39" s="40"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
@@ -5124,70 +5185,118 @@
       <c r="B40" s="30">
         <v>46010</v>
       </c>
-      <c r="C40" s="31"/>
-      <c r="D40" s="32"/>
-      <c r="E40" s="33"/>
+      <c r="C40" s="31">
+        <v>1</v>
+      </c>
+      <c r="D40" s="32">
+        <v>30</v>
+      </c>
+      <c r="E40" s="33" t="s">
+        <v>17</v>
+      </c>
       <c r="F40" s="22"/>
       <c r="G40" s="39"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="63" t="str">
+      <c r="A41" s="63">
         <f>IF(ISBLANK(B41),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B41))</f>
-        <v/>
-      </c>
-      <c r="B41" s="34"/>
+        <v>51</v>
+      </c>
+      <c r="B41" s="34">
+        <v>46010</v>
+      </c>
       <c r="C41" s="35"/>
-      <c r="D41" s="36"/>
-      <c r="E41" s="37"/>
-      <c r="F41" s="22"/>
+      <c r="D41" s="36">
+        <v>40</v>
+      </c>
+      <c r="E41" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F41" s="22" t="s">
+        <v>61</v>
+      </c>
       <c r="G41" s="40"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" s="62" t="str">
+      <c r="A42" s="62">
         <f>IF(ISBLANK(B42),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B42))</f>
-        <v/>
-      </c>
-      <c r="B42" s="30"/>
+        <v>51</v>
+      </c>
+      <c r="B42" s="30">
+        <v>46010</v>
+      </c>
       <c r="C42" s="31"/>
-      <c r="D42" s="32"/>
-      <c r="E42" s="33"/>
-      <c r="F42" s="22"/>
+      <c r="D42" s="32">
+        <v>5</v>
+      </c>
+      <c r="E42" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="F42" s="22" t="s">
+        <v>30</v>
+      </c>
       <c r="G42" s="39"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="63" t="str">
+      <c r="A43" s="63">
         <f>IF(ISBLANK(B43),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B43))</f>
-        <v/>
-      </c>
-      <c r="B43" s="34"/>
-      <c r="C43" s="35"/>
-      <c r="D43" s="36"/>
-      <c r="E43" s="37"/>
-      <c r="F43" s="22"/>
+        <v>2</v>
+      </c>
+      <c r="B43" s="34">
+        <v>46031</v>
+      </c>
+      <c r="C43" s="35">
+        <v>1</v>
+      </c>
+      <c r="D43" s="36">
+        <v>35</v>
+      </c>
+      <c r="E43" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F43" s="22" t="s">
+        <v>62</v>
+      </c>
       <c r="G43" s="40"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="62" t="str">
+      <c r="A44" s="62">
         <f>IF(ISBLANK(B44),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B44))</f>
-        <v/>
-      </c>
-      <c r="B44" s="30"/>
+        <v>2</v>
+      </c>
+      <c r="B44" s="30">
+        <v>46031</v>
+      </c>
       <c r="C44" s="31"/>
-      <c r="D44" s="32"/>
-      <c r="E44" s="33"/>
-      <c r="F44" s="22"/>
+      <c r="D44" s="32">
+        <v>30</v>
+      </c>
+      <c r="E44" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F44" s="22" t="s">
+        <v>63</v>
+      </c>
       <c r="G44" s="39"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" s="63" t="str">
+      <c r="A45" s="63">
         <f>IF(ISBLANK(B45),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B45))</f>
-        <v/>
-      </c>
-      <c r="B45" s="34"/>
+        <v>2</v>
+      </c>
+      <c r="B45" s="34">
+        <v>46031</v>
+      </c>
       <c r="C45" s="35"/>
-      <c r="D45" s="36"/>
-      <c r="E45" s="37"/>
-      <c r="F45" s="22"/>
+      <c r="D45" s="36">
+        <v>10</v>
+      </c>
+      <c r="E45" s="37" t="s">
+        <v>13</v>
+      </c>
+      <c r="F45" s="22" t="s">
+        <v>30</v>
+      </c>
       <c r="G45" s="40"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
@@ -11205,15 +11314,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>440</v>
+        <v>605</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>500</v>
+        <v>725</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11221,11 +11330,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>8 h 20 min</v>
+        <v>12 h 05 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.64935064935064934</v>
+        <v>0.65610859728506787</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11283,11 +11392,11 @@
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
-        <v>105</v>
+        <v>125</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>225</v>
+        <v>245</v>
       </c>
       <c r="E9" s="77" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11295,11 +11404,11 @@
       </c>
       <c r="F9" s="74" t="str">
         <f t="shared" si="1"/>
-        <v>3 h 45 min</v>
+        <v>4 h 05 min</v>
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.29220779220779219</v>
+        <v>0.22171945701357465</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11316,26 +11425,26 @@
     <row r="10" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E10,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="B10">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E10,'Journal de travail'!$D$7:$D$532)</f>
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="C10">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>135</v>
       </c>
       <c r="E10" s="78" t="s">
         <v>17</v>
       </c>
       <c r="F10" s="79" t="str">
         <f t="shared" ref="F10" si="4">QUOTIENT(SUM(A10:B10),60)&amp;" h "&amp;TEXT(MOD(SUM(A10:B10),60), "00")&amp;" min"</f>
-        <v>0 h 45 min</v>
+        <v>2 h 15 min</v>
       </c>
       <c r="G10" s="80">
         <f>SUM(A10:B10)/$C$11</f>
-        <v>5.844155844155844E-2</v>
+        <v>0.12217194570135746</v>
       </c>
       <c r="L10" s="69" t="s">
         <v>17</v>
@@ -11351,26 +11460,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>180</v>
+        <v>300</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>590</v>
+        <v>805</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>770</v>
+        <v>1105</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>28</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>12 h 50 min</v>
+        <v>18 h 25 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.1425925925925926</v>
+        <v>0.20462962962962963</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>28</v>
@@ -11409,14 +11518,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11615,21 +11722,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
-    <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11654,9 +11760,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
+    <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>